<commit_message>
Update Privacy News Dashboard snapshot (2026-07-20 10:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/kisa.xlsx
+++ b/docs/snapshot/downloads/kisa.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,7 +476,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>11331</t>
+          <t>14431</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -486,22 +486,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -517,19 +517,19 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>10981</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -539,17 +539,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
+          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -559,7 +559,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -574,49 +574,49 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>10943</t>
+          <t>14444</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1493</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -627,19 +627,19 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>10663</t>
+          <t>11331</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -649,22 +649,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
+          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -675,57 +675,61 @@
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>9805</t>
+          <t>10981</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
+          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -733,19 +737,19 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>9691</t>
+          <t>10943</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -755,87 +759,83 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
+          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>9321</t>
+          <t>10663</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
+          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -843,19 +843,19 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>8871</t>
+          <t>9805</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -865,22 +865,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
+          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -891,24 +891,24 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>6685</t>
+          <t>9691</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -918,22 +918,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
+          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -944,77 +944,81 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>6571</t>
+          <t>9321</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
+          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>5591</t>
+          <t>8871</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1024,22 +1028,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
+          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1055,44 +1059,44 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>6685</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
+          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1103,49 +1107,49 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>4762</t>
+          <t>6571</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AI 보안 위협 대응 매뉴얼</t>
+          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1153,56 +1157,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>4761</t>
+          <t>5591</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AI 보안 레드티밍 가이드</t>
+          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1210,56 +1210,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>961</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
+          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1275,34 +1271,34 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>4762</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
+          <t>AI 보안 위협 대응 매뉴얼</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1312,15 +1308,19 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -1328,44 +1328,44 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>4761</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
+          <t>AI 보안 레드티밍 가이드</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1373,52 +1373,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
+          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>191</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1426,68 +1430,60 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3867</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
+          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -1495,44 +1491,44 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4111</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1477</t>
+          <t>959</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
+          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1543,49 +1539,49 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
+          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1593,7 +1589,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -1613,7 +1613,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1623,27 +1623,27 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
+          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1670,22 +1670,22 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1477</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026년 IoT 보안인증 교육과정 안내</t>
+          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1695,19 +1695,15 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>386</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -1727,32 +1723,32 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
+          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>362</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,7 +1776,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1790,27 +1786,27 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>522</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1837,40 +1833,44 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
+          <t>2026년 IoT 보안인증 교육과정 안내</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2264</t>
+          <t>652</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -1878,44 +1878,44 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>958</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
+          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>76426</t>
+          <t>818</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1926,49 +1926,49 @@
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>956</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
+          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>55906</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1976,52 +1976,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>957</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>55329</t>
+          <t>2264</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2032,49 +2036,49 @@
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>955</t>
+          <t>958</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
+          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>34467</t>
+          <t>76426</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2102,89 +2106,85 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>956</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
+          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2945</t>
+          <t>55906</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>957</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
+          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>5048</t>
+          <t>55329</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2192,56 +2192,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>954</t>
+          <t>955</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>145255</t>
+          <t>34467</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2269,85 +2265,89 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>26576</t>
+          <t>2945</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>952</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
+          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>34290</t>
+          <t>5048</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2355,52 +2355,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>951</t>
+          <t>954</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>184573</t>
+          <t>145255</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2428,32 +2432,32 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>953</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>51749</t>
+          <t>26576</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2481,32 +2485,32 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>949</t>
+          <t>952</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>78439</t>
+          <t>34290</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2526,6 +2530,222 @@
         </is>
       </c>
       <c r="K39" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>951</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>184573</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>14403</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>공지</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>6587</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>공지사항</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>950</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>51749</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>949</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>78439</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-08-13 10:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/kisa.xlsx
+++ b/docs/snapshot/downloads/kisa.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K74"/>
+  <dimension ref="A1:K75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,32 +476,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>34071</t>
+          <t>34081</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>978</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>"예방 넘어 대응·복구까지" 랜섬웨어 전주기 대응 방안 논의한다</t>
+          <t>2026년 하반기 정보보호 전문서비스 기업 지정에 관한 공고</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2626&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3742&amp;page=1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -509,42 +509,46 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-08-13 09:16:35.989405+09:00</t>
+          <t>2026-08-13 09:31:24.927741+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-08-13 09:16:35.989405+09:00</t>
+          <t>2026-08-13 09:31:24.927741+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>33789</t>
+          <t>34071</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>978</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 21회차 교육생 모집(~9.11)</t>
+          <t>"예방 넘어 대응·복구까지" 랜섬웨어 전주기 대응 방안 논의한다</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3741&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2626&amp;page=1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -554,35 +558,35 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-08-12 16:01:25.579701+09:00</t>
+          <t>2026-08-13 09:16:35.989405+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-08-12 16:01:25.579701+09:00</t>
+          <t>2026-08-13 09:16:35.989405+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>33749</t>
+          <t>33789</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -592,12 +596,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026년도 블록체인 유공 포상 계획 공고 안내(~9.21 15:00 마감)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 21회차 교육생 모집(~9.11)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3740&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3741&amp;page=1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -607,12 +611,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -623,44 +627,44 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-08-12 15:31:25.306307+09:00</t>
+          <t>2026-08-12 16:01:25.579701+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-08-12 15:31:25.306307+09:00</t>
+          <t>2026-08-12 16:01:25.579701+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>31741</t>
+          <t>33749</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026년 블록체인 수요-공급 협의체 (ABLE) 정례세미나 개최 안내(8.13.목)</t>
+          <t>2026년도 블록체인 유공 포상 계획 공고 안내(~9.21 15:00 마감)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3739&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3740&amp;page=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -668,11 +672,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -680,52 +680,56 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-08-10 11:01:30.246604+09:00</t>
+          <t>2026-08-12 15:31:25.306307+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-08-10 11:01:30.246604+09:00</t>
+          <t>2026-08-12 15:31:25.306307+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>29768</t>
+          <t>31741</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026년 블록체인 신뢰인프라(K-BTF) 활용·확산사업 공모 사전예고</t>
+          <t>2026년 블록체인 수요-공급 협의체 (ABLE) 정례세미나 개최 안내(8.13.목)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3738&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3739&amp;page=1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>13</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -733,19 +737,19 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-08-07 17:01:29.954014+09:00</t>
+          <t>2026-08-10 11:01:30.246604+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-08-07 17:01:29.954014+09:00</t>
+          <t>2026-08-10 11:01:30.246604+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>29728</t>
+          <t>29768</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -755,12 +759,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026년도 블록체인 산업 실태조사 실시 및 협조 안내</t>
+          <t>2026년 블록체인 신뢰인프라(K-BTF) 활용·확산사업 공모 사전예고</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3737&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3738&amp;page=1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -770,7 +774,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -786,19 +790,19 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-08-07 16:31:30.938844+09:00</t>
+          <t>2026-08-07 17:01:29.954014+09:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-08-07 16:31:30.938844+09:00</t>
+          <t>2026-08-07 17:01:29.954014+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>28711</t>
+          <t>29728</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -808,50 +812,50 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원-나주시, 고교생 개인정보·정보보호 진로 탐색 지원</t>
+          <t>2026년도 블록체인 산업 실태조사 실시 및 협조 안내</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2625&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3737&amp;page=1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-08-06 14:01:34.968573+09:00</t>
+          <t>2026-08-07 16:31:30.938844+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-08-06 14:01:34.968573+09:00</t>
+          <t>2026-08-07 16:31:30.938844+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>27551</t>
+          <t>28711</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -861,22 +865,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 기업 맞춤형 사이버 위협 알림 서비스 개시</t>
+          <t>한국인터넷진흥원-나주시, 고교생 개인정보·정보보호 진로 탐색 지원</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2624&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2625&amp;page=1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>101</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -892,44 +896,44 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-08-05 09:46:34.063806+09:00</t>
+          <t>2026-08-06 14:01:34.968573+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-08-05 09:46:34.063806+09:00</t>
+          <t>2026-08-06 14:01:34.968573+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>27511</t>
+          <t>27551</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>975</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 기관장 주도 국민 체감 성과 혁신 체계 가동</t>
+          <t>한국인터넷진흥원, 기업 맞춤형 사이버 위협 알림 서비스 개시</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2623&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2624&amp;page=1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>263</t>
+          <t>101</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -945,34 +949,34 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-08-05 09:16:33.823896+09:00</t>
+          <t>2026-08-05 09:46:34.063806+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-08-05 09:16:33.823896+09:00</t>
+          <t>2026-08-05 09:46:34.063806+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>27268</t>
+          <t>27511</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>975</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>양자내성암호 국제 표준화 동향 분석</t>
+          <t>한국인터넷진흥원, 기관장 주도 국민 체감 성과 혁신 체계 가동</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3736&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2623&amp;page=1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -982,7 +986,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>263</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -993,24 +997,24 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-08-04 16:31:26.502205+09:00</t>
+          <t>2026-08-05 09:16:33.823896+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-08-04 16:31:26.502205+09:00</t>
+          <t>2026-08-05 09:16:33.823896+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>27128</t>
+          <t>27268</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1020,12 +1024,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 20회차 교육생 모집(~9.4)</t>
+          <t>양자내성암호 국제 표준화 동향 분석</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3735&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3736&amp;page=1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1035,12 +1039,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
@@ -1051,19 +1055,19 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-08-04 14:46:28.764255+09:00</t>
+          <t>2026-08-04 16:31:26.502205+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-08-04 14:46:28.764255+09:00</t>
+          <t>2026-08-04 16:31:26.502205+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>26211</t>
+          <t>27128</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1073,50 +1077,50 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 암호모듈검증 위한 시험 전문인력 양성</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 20회차 교육생 모집(~9.4)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2622&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3735&amp;page=1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>273</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-08-03 13:31:41.722921+09:00</t>
+          <t>2026-08-04 14:46:28.764255+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-08-03 13:31:41.722921+09:00</t>
+          <t>2026-08-04 14:46:28.764255+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>26188</t>
+          <t>26211</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1126,12 +1130,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026년 8차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(8월 추천) (~8.21(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 암호모듈검증 위한 시험 전문인력 양성</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3734&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2622&amp;page=1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1141,7 +1145,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>273</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1152,24 +1156,24 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-08-03 13:16:30.325331+09:00</t>
+          <t>2026-08-03 13:31:41.722921+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-08-03 13:16:30.325331+09:00</t>
+          <t>2026-08-03 13:31:41.722921+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>25891</t>
+          <t>26188</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1179,12 +1183,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 지역 상생 3대 사업 참여자 모집</t>
+          <t>2026년 8차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(8월 추천) (~8.21(금) 18시까지)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2621&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3734&amp;page=1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1194,7 +1198,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1205,39 +1209,39 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-08-03 09:31:46.854132+09:00</t>
+          <t>2026-08-03 13:16:30.325331+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-08-03 09:31:46.854132+09:00</t>
+          <t>2026-08-03 13:16:30.325331+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>25864</t>
+          <t>25891</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026년 전남광주통합특별시 소상공인·사회적경제기업 판로 확대 지원기업 선발 안내(~8.14)</t>
+          <t>한국인터넷진흥원, 지역 상생 3대 사업 참여자 모집</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3730&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2621&amp;page=1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1247,7 +1251,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>80</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1255,31 +1259,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-08-03 09:16:35.817723+09:00</t>
+          <t>2026-08-03 09:31:46.854132+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-08-03 09:16:35.817723+09:00</t>
+          <t>2026-08-03 09:31:46.854132+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>25863</t>
+          <t>25864</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1289,12 +1289,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026년 전남광주통합특별시 지역문제 해결 프로젝트 공모전 개최 안내(~8.21)</t>
+          <t>2026년 전남광주통합특별시 소상공인·사회적경제기업 판로 확대 지원기업 선발 안내(~8.14)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3731&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3730&amp;page=1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1304,7 +1304,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1336,7 +1336,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>25862</t>
+          <t>25863</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1346,12 +1346,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026년 한국인터넷진흥원 지역공부방 참여 대학생 장학금 지원자 모집 안내(~8.28)</t>
+          <t>2026년 전남광주통합특별시 지역문제 해결 프로젝트 공모전 개최 안내(~8.21)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3732&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3731&amp;page=1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1361,7 +1361,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1393,7 +1393,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>25861</t>
+          <t>25862</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1403,12 +1403,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026년 암호모듈 시험자 양성교육 및 필기시험 안내(8.3~8.21)</t>
+          <t>2026년 한국인터넷진흥원 지역공부방 참여 대학생 장학금 지원자 모집 안내(~8.28)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3733&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3732&amp;page=1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1450,7 +1450,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>23221</t>
+          <t>25861</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1460,22 +1460,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026년 블록체인 기업성장허브 입주기업 모집(~8월 27일(목) 16:00까지)</t>
+          <t>2026년 암호모듈 시험자 양성교육 및 필기시험 안내(8.3~8.21)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3729&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3733&amp;page=1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1495,52 +1495,56 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-30 17:16:54.540202+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-30 17:16:54.540202+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>22504</t>
+          <t>23221</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 19회차 교육생 모집(~8.28)</t>
+          <t>2026년 블록체인 기업성장허브 입주기업 모집(~8월 27일(목) 16:00까지)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3728&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3729&amp;page=1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -1548,19 +1552,19 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-29 18:32:00.075123+09:00</t>
+          <t>2026-07-30 17:16:54.540202+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-29 18:32:00.075123+09:00</t>
+          <t>2026-07-30 17:16:54.540202+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>22464</t>
+          <t>22504</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1570,12 +1574,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026년 연계정보 이용기관 안전조치 실태점검 2차 설명회 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 19회차 교육생 모집(~8.28)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3727&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3728&amp;page=1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1585,7 +1589,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1601,19 +1605,19 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-29 18:01:59.875668+09:00</t>
+          <t>2026-07-29 18:32:00.075123+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-29 18:01:59.875668+09:00</t>
+          <t>2026-07-29 18:32:00.075123+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>20771</t>
+          <t>22464</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1623,50 +1627,50 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
+          <t>2026년 연계정보 이용기관 안전조치 실태점검 2차 설명회 개최</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3727&amp;page=1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>20191</t>
+          <t>20771</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1676,12 +1680,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
+          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1691,7 +1695,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>287</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1707,34 +1711,34 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>20061</t>
+          <t>20191</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
+          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1744,7 +1748,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>246</t>
+          <t>287</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1752,64 +1756,64 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>16785</t>
+          <t>20061</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>1496</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
+          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>246</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -1817,34 +1821,34 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>16784</t>
+          <t>16785</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1497</t>
+          <t>1496</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1854,7 +1858,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>236</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1882,22 +1886,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>16781</t>
+          <t>16784</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1497</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1907,7 +1911,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>260</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1915,11 +1919,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -1939,22 +1939,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>16691</t>
+          <t>16781</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1964,35 +1964,39 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>278</t>
+          <t>242</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>16464</t>
+          <t>16691</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2002,12 +2006,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
+          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2017,35 +2021,35 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>278</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>16051</t>
+          <t>16464</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2055,12 +2059,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
+          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2070,35 +2074,35 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>14611</t>
+          <t>16051</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2108,22 +2112,22 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
+          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>233</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2139,19 +2143,19 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>14431</t>
+          <t>14611</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2161,12 +2165,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2176,7 +2180,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2192,34 +2196,34 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>14431</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2229,7 +2233,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2237,56 +2241,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>14444</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>1493</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2294,7 +2294,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -2302,34 +2306,34 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>11331</t>
+          <t>14444</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1493</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2339,7 +2343,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2350,96 +2354,92 @@
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>10981</t>
+          <t>11331</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
+          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>10943</t>
+          <t>10981</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
+          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2449,7 +2449,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2457,7 +2457,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I38" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -2465,19 +2469,19 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>10663</t>
+          <t>10943</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2487,12 +2491,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
+          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2502,12 +2506,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H39" t="inlineStr"/>
@@ -2518,19 +2522,19 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>9805</t>
+          <t>10663</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2540,22 +2544,22 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
+          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2571,19 +2575,19 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>9691</t>
+          <t>9805</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2593,12 +2597,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
+          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2608,7 +2612,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2619,96 +2623,92 @@
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>9321</t>
+          <t>9691</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
+          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>8871</t>
+          <t>9321</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
+          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2718,35 +2718,39 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>6685</t>
+          <t>8871</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2756,22 +2760,22 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
+          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2782,24 +2786,24 @@
       <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>6571</t>
+          <t>6685</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2809,12 +2813,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
+          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2824,7 +2828,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2835,24 +2839,24 @@
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>5591</t>
+          <t>6571</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2862,22 +2866,22 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
+          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2893,44 +2897,44 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>5591</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
+          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2946,44 +2950,44 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>4762</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>961</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>AI 보안 위협 대응 매뉴얼</t>
+          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2991,31 +2995,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>4761</t>
+          <t>4762</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -3025,12 +3025,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>AI 보안 레드티밍 가이드</t>
+          <t>AI 보안 위협 대응 매뉴얼</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -3040,7 +3040,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -3072,22 +3072,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>4761</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
+          <t>AI 보안 레드티밍 가이드</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -3097,7 +3097,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3105,27 +3105,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3135,12 +3139,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
+          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -3150,113 +3154,113 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>191</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>3867</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
+          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4111</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>959</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3264,31 +3268,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3298,12 +3298,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
+          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -3313,7 +3313,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -3345,32 +3345,32 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>1477</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
+          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -3378,7 +3378,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr"/>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I55" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -3398,22 +3402,22 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>1477</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
+          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3423,7 +3427,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>386</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3451,22 +3455,22 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
+          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -3476,19 +3480,15 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>362</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -3508,7 +3508,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3518,12 +3518,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026년 IoT 보안인증 교육과정 안내</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -3533,7 +3533,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>522</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -3565,40 +3565,44 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
+          <t>2026년 IoT 보안인증 교육과정 안내</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>652</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I59" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -3618,22 +3622,22 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
+          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3643,7 +3647,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>818</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -3651,11 +3655,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -3675,32 +3675,32 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
+          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>2264</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3708,7 +3708,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr"/>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I61" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -3716,34 +3720,34 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>958</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3753,7 +3757,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>76426</t>
+          <t>2264</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -3764,49 +3768,49 @@
       <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>956</t>
+          <t>958</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
+          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>55906</t>
+          <t>76426</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3834,22 +3838,22 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>957</t>
+          <t>956</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
+          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3859,7 +3863,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>55329</t>
+          <t>55906</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3887,32 +3891,32 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>955</t>
+          <t>957</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
+          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>34467</t>
+          <t>55329</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3940,22 +3944,22 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>955</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
+          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3965,39 +3969,35 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>2945</t>
+          <t>34467</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -4007,27 +4007,27 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>5048</t>
+          <t>2945</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -4054,32 +4054,32 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>954</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>145255</t>
+          <t>5048</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -4087,52 +4087,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr"/>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>954</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>26576</t>
+          <t>145255</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -4160,32 +4164,32 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>952</t>
+          <t>953</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
+          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>34290</t>
+          <t>26576</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -4213,32 +4217,32 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>951</t>
+          <t>952</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>184573</t>
+          <t>34290</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -4266,32 +4270,32 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>14403</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>951</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>6587</t>
+          <t>184573</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -4299,46 +4303,42 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H72" t="inlineStr"/>
       <c r="I72" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>14403</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -4348,7 +4348,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>51749</t>
+          <t>6587</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -4356,52 +4356,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr"/>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>949</t>
+          <t>950</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>78439</t>
+          <t>51749</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -4421,6 +4425,59 @@
         </is>
       </c>
       <c r="K74" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>949</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>78439</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-08-13 18:20:02 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/kisa.xlsx
+++ b/docs/snapshot/downloads/kisa.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K75"/>
+  <dimension ref="A1:K76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,22 +476,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>34081</t>
+          <t>34750</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026년 하반기 정보보호 전문서비스 기업 지정에 관한 공고</t>
+          <t>｢2026 블록체인 진흥주간｣ 전시부스 참가기업 모집 공고(~9.14)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3742&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3743&amp;page=1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -501,7 +501,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -509,11 +509,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -521,44 +517,44 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-08-13 09:31:24.927741+09:00</t>
+          <t>2026-08-13 17:46:21.938331+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-08-13 09:31:24.927741+09:00</t>
+          <t>2026-08-13 17:46:21.938331+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>34071</t>
+          <t>34081</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>978</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>"예방 넘어 대응·복구까지" 랜섬웨어 전주기 대응 방안 논의한다</t>
+          <t>2026년 하반기 정보보호 전문서비스 기업 지정에 관한 공고</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2626&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3742&amp;page=1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -566,42 +562,46 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-08-13 09:16:35.989405+09:00</t>
+          <t>2026-08-13 09:31:24.927741+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-08-13 09:16:35.989405+09:00</t>
+          <t>2026-08-13 09:31:24.927741+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>33789</t>
+          <t>34071</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>978</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 21회차 교육생 모집(~9.11)</t>
+          <t>"예방 넘어 대응·복구까지" 랜섬웨어 전주기 대응 방안 논의한다</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3741&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2626&amp;page=1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -611,35 +611,35 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-08-12 16:01:25.579701+09:00</t>
+          <t>2026-08-13 09:16:35.989405+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-08-12 16:01:25.579701+09:00</t>
+          <t>2026-08-13 09:16:35.989405+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>33749</t>
+          <t>33789</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -649,12 +649,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026년도 블록체인 유공 포상 계획 공고 안내(~9.21 15:00 마감)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 21회차 교육생 모집(~9.11)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3740&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3741&amp;page=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -664,12 +664,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -680,44 +680,44 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-08-12 15:31:25.306307+09:00</t>
+          <t>2026-08-12 16:01:25.579701+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-08-12 15:31:25.306307+09:00</t>
+          <t>2026-08-12 16:01:25.579701+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>31741</t>
+          <t>33749</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026년 블록체인 수요-공급 협의체 (ABLE) 정례세미나 개최 안내(8.13.목)</t>
+          <t>2026년도 블록체인 유공 포상 계획 공고 안내(~9.21 15:00 마감)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3739&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3740&amp;page=1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -725,11 +725,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -737,52 +733,56 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-08-10 11:01:30.246604+09:00</t>
+          <t>2026-08-12 15:31:25.306307+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-08-10 11:01:30.246604+09:00</t>
+          <t>2026-08-12 15:31:25.306307+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>29768</t>
+          <t>31741</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026년 블록체인 신뢰인프라(K-BTF) 활용·확산사업 공모 사전예고</t>
+          <t>2026년 블록체인 수요-공급 협의체 (ABLE) 정례세미나 개최 안내(8.13.목)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3738&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3739&amp;page=1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>13</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -790,19 +790,19 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-08-07 17:01:29.954014+09:00</t>
+          <t>2026-08-10 11:01:30.246604+09:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-08-07 17:01:29.954014+09:00</t>
+          <t>2026-08-10 11:01:30.246604+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>29728</t>
+          <t>29768</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -812,12 +812,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026년도 블록체인 산업 실태조사 실시 및 협조 안내</t>
+          <t>2026년 블록체인 신뢰인프라(K-BTF) 활용·확산사업 공모 사전예고</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3737&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3738&amp;page=1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -843,19 +843,19 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-08-07 16:31:30.938844+09:00</t>
+          <t>2026-08-07 17:01:29.954014+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-08-07 16:31:30.938844+09:00</t>
+          <t>2026-08-07 17:01:29.954014+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>28711</t>
+          <t>29728</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -865,50 +865,50 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원-나주시, 고교생 개인정보·정보보호 진로 탐색 지원</t>
+          <t>2026년도 블록체인 산업 실태조사 실시 및 협조 안내</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2625&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3737&amp;page=1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-08-06 14:01:34.968573+09:00</t>
+          <t>2026-08-07 16:31:30.938844+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-08-06 14:01:34.968573+09:00</t>
+          <t>2026-08-07 16:31:30.938844+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>27551</t>
+          <t>28711</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -918,22 +918,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 기업 맞춤형 사이버 위협 알림 서비스 개시</t>
+          <t>한국인터넷진흥원-나주시, 고교생 개인정보·정보보호 진로 탐색 지원</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2624&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2625&amp;page=1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>101</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -949,44 +949,44 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-08-05 09:46:34.063806+09:00</t>
+          <t>2026-08-06 14:01:34.968573+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-08-05 09:46:34.063806+09:00</t>
+          <t>2026-08-06 14:01:34.968573+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>27511</t>
+          <t>27551</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>975</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 기관장 주도 국민 체감 성과 혁신 체계 가동</t>
+          <t>한국인터넷진흥원, 기업 맞춤형 사이버 위협 알림 서비스 개시</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2623&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2624&amp;page=1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>263</t>
+          <t>101</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1002,34 +1002,34 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-08-05 09:16:33.823896+09:00</t>
+          <t>2026-08-05 09:46:34.063806+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-08-05 09:16:33.823896+09:00</t>
+          <t>2026-08-05 09:46:34.063806+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>27268</t>
+          <t>27511</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>975</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>양자내성암호 국제 표준화 동향 분석</t>
+          <t>한국인터넷진흥원, 기관장 주도 국민 체감 성과 혁신 체계 가동</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3736&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2623&amp;page=1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>263</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1050,24 +1050,24 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-08-04 16:31:26.502205+09:00</t>
+          <t>2026-08-05 09:16:33.823896+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-08-04 16:31:26.502205+09:00</t>
+          <t>2026-08-05 09:16:33.823896+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>27128</t>
+          <t>27268</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1077,12 +1077,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 20회차 교육생 모집(~9.4)</t>
+          <t>양자내성암호 국제 표준화 동향 분석</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3735&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3736&amp;page=1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1092,12 +1092,12 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -1108,19 +1108,19 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-08-04 14:46:28.764255+09:00</t>
+          <t>2026-08-04 16:31:26.502205+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-08-04 14:46:28.764255+09:00</t>
+          <t>2026-08-04 16:31:26.502205+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>26211</t>
+          <t>27128</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1130,50 +1130,50 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 암호모듈검증 위한 시험 전문인력 양성</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 20회차 교육생 모집(~9.4)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2622&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3735&amp;page=1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>273</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-08-03 13:31:41.722921+09:00</t>
+          <t>2026-08-04 14:46:28.764255+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-08-03 13:31:41.722921+09:00</t>
+          <t>2026-08-04 14:46:28.764255+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>26188</t>
+          <t>26211</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1183,12 +1183,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026년 8차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(8월 추천) (~8.21(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 암호모듈검증 위한 시험 전문인력 양성</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3734&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2622&amp;page=1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>273</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1209,24 +1209,24 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-08-03 13:16:30.325331+09:00</t>
+          <t>2026-08-03 13:31:41.722921+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-08-03 13:16:30.325331+09:00</t>
+          <t>2026-08-03 13:31:41.722921+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>25891</t>
+          <t>26188</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1236,12 +1236,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 지역 상생 3대 사업 참여자 모집</t>
+          <t>2026년 8차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(8월 추천) (~8.21(금) 18시까지)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2621&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3734&amp;page=1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1262,39 +1262,39 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-08-03 09:31:46.854132+09:00</t>
+          <t>2026-08-03 13:16:30.325331+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-08-03 09:31:46.854132+09:00</t>
+          <t>2026-08-03 13:16:30.325331+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>25864</t>
+          <t>25891</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026년 전남광주통합특별시 소상공인·사회적경제기업 판로 확대 지원기업 선발 안내(~8.14)</t>
+          <t>한국인터넷진흥원, 지역 상생 3대 사업 참여자 모집</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3730&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2621&amp;page=1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1304,7 +1304,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>80</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1312,31 +1312,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-08-03 09:16:35.817723+09:00</t>
+          <t>2026-08-03 09:31:46.854132+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-08-03 09:16:35.817723+09:00</t>
+          <t>2026-08-03 09:31:46.854132+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>25863</t>
+          <t>25864</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1346,12 +1342,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026년 전남광주통합특별시 지역문제 해결 프로젝트 공모전 개최 안내(~8.21)</t>
+          <t>2026년 전남광주통합특별시 소상공인·사회적경제기업 판로 확대 지원기업 선발 안내(~8.14)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3731&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3730&amp;page=1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1361,7 +1357,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1393,7 +1389,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>25862</t>
+          <t>25863</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1403,12 +1399,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026년 한국인터넷진흥원 지역공부방 참여 대학생 장학금 지원자 모집 안내(~8.28)</t>
+          <t>2026년 전남광주통합특별시 지역문제 해결 프로젝트 공모전 개최 안내(~8.21)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3732&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3731&amp;page=1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1418,7 +1414,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1450,7 +1446,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>25861</t>
+          <t>25862</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1460,12 +1456,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026년 암호모듈 시험자 양성교육 및 필기시험 안내(8.3~8.21)</t>
+          <t>2026년 한국인터넷진흥원 지역공부방 참여 대학생 장학금 지원자 모집 안내(~8.28)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3733&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3732&amp;page=1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1475,7 +1471,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1507,7 +1503,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>23221</t>
+          <t>25861</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1517,22 +1513,22 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026년 블록체인 기업성장허브 입주기업 모집(~8월 27일(목) 16:00까지)</t>
+          <t>2026년 암호모듈 시험자 양성교육 및 필기시험 안내(8.3~8.21)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3729&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3733&amp;page=1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1552,52 +1548,56 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-30 17:16:54.540202+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-30 17:16:54.540202+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>22504</t>
+          <t>23221</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 19회차 교육생 모집(~8.28)</t>
+          <t>2026년 블록체인 기업성장허브 입주기업 모집(~8월 27일(목) 16:00까지)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3728&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3729&amp;page=1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -1605,19 +1605,19 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-07-29 18:32:00.075123+09:00</t>
+          <t>2026-07-30 17:16:54.540202+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-29 18:32:00.075123+09:00</t>
+          <t>2026-07-30 17:16:54.540202+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>22464</t>
+          <t>22504</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1627,12 +1627,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026년 연계정보 이용기관 안전조치 실태점검 2차 설명회 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 19회차 교육생 모집(~8.28)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3727&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3728&amp;page=1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1642,7 +1642,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1658,19 +1658,19 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-07-29 18:01:59.875668+09:00</t>
+          <t>2026-07-29 18:32:00.075123+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-29 18:01:59.875668+09:00</t>
+          <t>2026-07-29 18:32:00.075123+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>20771</t>
+          <t>22464</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1680,50 +1680,50 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
+          <t>2026년 연계정보 이용기관 안전조치 실태점검 2차 설명회 개최</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3727&amp;page=1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>20191</t>
+          <t>20771</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1733,12 +1733,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
+          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1748,7 +1748,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>287</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1764,34 +1764,34 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>20061</t>
+          <t>20191</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
+          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>246</t>
+          <t>287</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1809,64 +1809,64 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>16785</t>
+          <t>20061</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1496</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
+          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>246</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -1874,34 +1874,34 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>16784</t>
+          <t>16785</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>1497</t>
+          <t>1496</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1911,7 +1911,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>236</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1939,22 +1939,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>16781</t>
+          <t>16784</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1497</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>260</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1972,11 +1972,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -1996,22 +1992,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>16691</t>
+          <t>16781</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2021,35 +2017,39 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>278</t>
+          <t>242</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>16464</t>
+          <t>16691</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2059,12 +2059,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
+          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2074,35 +2074,35 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>278</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>16051</t>
+          <t>16464</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2112,12 +2112,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
+          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2127,35 +2127,35 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>14611</t>
+          <t>16051</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2165,22 +2165,22 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
+          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>233</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2196,19 +2196,19 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>14431</t>
+          <t>14611</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2218,12 +2218,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2249,34 +2249,34 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>14431</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2286,7 +2286,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2294,56 +2294,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>14444</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>1493</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2351,7 +2347,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -2359,34 +2359,34 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>11331</t>
+          <t>14444</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1493</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2396,7 +2396,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2407,96 +2407,92 @@
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>10981</t>
+          <t>11331</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
+          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>10943</t>
+          <t>10981</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
+          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2506,7 +2502,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2514,7 +2510,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -2522,19 +2522,19 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>10663</t>
+          <t>10943</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2544,12 +2544,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
+          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2559,12 +2559,12 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H40" t="inlineStr"/>
@@ -2575,19 +2575,19 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>9805</t>
+          <t>10663</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2597,22 +2597,22 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
+          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2628,19 +2628,19 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>9691</t>
+          <t>9805</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2650,12 +2650,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
+          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2676,96 +2676,92 @@
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>9321</t>
+          <t>9691</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
+          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>8871</t>
+          <t>9321</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
+          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2775,35 +2771,39 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>6685</t>
+          <t>8871</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2813,22 +2813,22 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
+          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2839,24 +2839,24 @@
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>6571</t>
+          <t>6685</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2866,12 +2866,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
+          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2881,7 +2881,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2892,24 +2892,24 @@
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>5591</t>
+          <t>6571</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2919,22 +2919,22 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
+          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2950,44 +2950,44 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>5591</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
+          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3003,44 +3003,44 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>4762</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>961</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>AI 보안 위협 대응 매뉴얼</t>
+          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -3048,31 +3048,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>4761</t>
+          <t>4762</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3082,12 +3078,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>AI 보안 레드티밍 가이드</t>
+          <t>AI 보안 위협 대응 매뉴얼</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -3097,7 +3093,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3129,22 +3125,22 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>4761</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
+          <t>AI 보안 레드티밍 가이드</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -3154,7 +3150,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3162,27 +3158,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -3192,12 +3192,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
+          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -3207,113 +3207,113 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>191</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>3867</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
+          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4111</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>959</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -3321,31 +3321,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3355,12 +3351,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
+          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -3370,7 +3366,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -3402,32 +3398,32 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>1477</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
+          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3435,7 +3431,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr"/>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I56" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -3455,22 +3455,22 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>1477</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
+          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -3480,7 +3480,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>386</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3508,22 +3508,22 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
+          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -3533,19 +3533,15 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>362</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -3565,7 +3561,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3575,12 +3571,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026년 IoT 보안인증 교육과정 안내</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -3590,7 +3586,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>522</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -3622,40 +3618,44 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
+          <t>2026년 IoT 보안인증 교육과정 안내</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>652</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I60" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -3675,22 +3675,22 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
+          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>818</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3708,11 +3708,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -3732,32 +3728,32 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
+          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>2264</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -3765,7 +3761,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr"/>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I62" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -3773,34 +3773,34 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>958</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3810,7 +3810,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>76426</t>
+          <t>2264</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3821,49 +3821,49 @@
       <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>956</t>
+          <t>958</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
+          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>55906</t>
+          <t>76426</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3891,22 +3891,22 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>957</t>
+          <t>956</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
+          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3916,7 +3916,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>55329</t>
+          <t>55906</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3944,32 +3944,32 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>955</t>
+          <t>957</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
+          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>34467</t>
+          <t>55329</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3997,22 +3997,22 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>955</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
+          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -4022,39 +4022,35 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>2945</t>
+          <t>34467</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -4064,27 +4060,27 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>5048</t>
+          <t>2945</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -4111,32 +4107,32 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>954</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>145255</t>
+          <t>5048</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -4144,52 +4140,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr"/>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>954</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>26576</t>
+          <t>145255</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -4217,32 +4217,32 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>952</t>
+          <t>953</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
+          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>34290</t>
+          <t>26576</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -4270,32 +4270,32 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>951</t>
+          <t>952</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>184573</t>
+          <t>34290</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -4323,32 +4323,32 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>14403</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>951</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>6587</t>
+          <t>184573</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -4356,46 +4356,42 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H73" t="inlineStr"/>
       <c r="I73" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>14403</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -4405,7 +4401,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>51749</t>
+          <t>6587</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -4413,52 +4409,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr"/>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>949</t>
+          <t>950</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>78439</t>
+          <t>51749</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -4478,6 +4478,59 @@
         </is>
       </c>
       <c r="K75" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>949</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>78439</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
         <is>
           <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-08-27 11:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/kisa.xlsx
+++ b/docs/snapshot/downloads/kisa.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K85"/>
+  <dimension ref="A1:K86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,32 +476,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>45191</t>
+          <t>45681</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 아·태 지역 사이버공격 대응 공동 훈련 실시</t>
+          <t>싱가포르 현지 진출 지원 국내 블록체인 기업 모집(~9.16(수) 14시)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2629&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3750&amp;page=1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -509,42 +509,46 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-08-26 15:01:47.261933+09:00</t>
+          <t>2026-08-27 11:01:31.314899+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-08-26 15:01:47.261933+09:00</t>
+          <t>2026-08-27 11:01:31.314899+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>44741</t>
+          <t>45191</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>[3차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~9/16)</t>
+          <t>한국인터넷진흥원, 아·태 지역 사이버공격 대응 공동 훈련 실시</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3749&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2629&amp;page=1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -554,7 +558,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -562,56 +566,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-08-26 09:31:36.427758+09:00</t>
+          <t>2026-08-26 15:01:47.261933+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-08-26 09:31:36.427758+09:00</t>
+          <t>2026-08-26 15:01:47.261933+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>44448</t>
+          <t>44741</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 공고</t>
+          <t>[3차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~9/16)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3748&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3749&amp;page=1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -619,7 +619,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -627,19 +631,19 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-08-25 16:01:39.626193+09:00</t>
+          <t>2026-08-26 09:31:36.427758+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-08-25 16:01:39.626193+09:00</t>
+          <t>2026-08-26 09:31:36.427758+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>43767</t>
+          <t>44448</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -649,27 +653,27 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 21회차 교육생 모집(~9.12)</t>
+          <t>정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 공고</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3747&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3748&amp;page=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -680,19 +684,19 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-08-24 17:46:42.254577+09:00</t>
+          <t>2026-08-25 16:01:39.626193+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-08-24 17:46:42.254577+09:00</t>
+          <t>2026-08-25 16:01:39.626193+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>43311</t>
+          <t>43767</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -702,12 +706,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>양자내성암호 전환, 어떻게 준비해야 할까?</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 21회차 교육생 모집(~9.12)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2627&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3747&amp;page=1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -717,50 +721,50 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-08-24 12:01:45.511381+09:00</t>
+          <t>2026-08-24 17:46:42.254577+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-08-24 12:01:45.511381+09:00</t>
+          <t>2026-08-24 17:46:42.254577+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>43301</t>
+          <t>43311</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 실무과정 교육생 모집(8.24~)</t>
+          <t>양자내성암호 전환, 어떻게 준비해야 할까?</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3746&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2627&amp;page=1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -770,7 +774,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -778,31 +782,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-08-24 12:01:36.271108+09:00</t>
+          <t>2026-08-24 12:01:45.511381+09:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-08-24 12:01:36.271108+09:00</t>
+          <t>2026-08-24 12:01:45.511381+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>41161</t>
+          <t>43301</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -812,27 +812,27 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>「블록체인 기업 맞춤형 보안 고도화 지원」 기업 모집(~8/31)</t>
+          <t>양자내성암호 전문교육 PQC 실무과정 교육생 모집(8.24~)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3745&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3746&amp;page=1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -847,34 +847,34 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-08-21 16:01:38.087170+09:00</t>
+          <t>2026-08-24 12:01:36.271108+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-08-21 16:01:38.087170+09:00</t>
+          <t>2026-08-24 12:01:36.271108+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>41086</t>
+          <t>41161</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026년도 인터넷거버넌스 민간전문가 APrIGF 및 IGF 참석자 모집</t>
+          <t>「블록체인 기업 맞춤형 보안 고도화 지원」 기업 모집(~8/31)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3744&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3745&amp;page=1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -884,15 +884,19 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -900,19 +904,19 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-08-21 15:01:32.139445+09:00</t>
+          <t>2026-08-21 16:01:38.087170+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-08-21 15:01:32.139445+09:00</t>
+          <t>2026-08-21 16:01:38.087170+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>34750</t>
+          <t>41086</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -922,22 +926,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>｢2026 블록체인 진흥주간｣ 전시부스 참가기업 모집 공고(~9.14)</t>
+          <t>2026년도 인터넷거버넌스 민간전문가 APrIGF 및 IGF 참석자 모집</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3743&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3744&amp;page=1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>59</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -953,34 +957,34 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-08-13 17:46:21.938331+09:00</t>
+          <t>2026-08-21 15:01:32.139445+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-08-13 17:46:21.938331+09:00</t>
+          <t>2026-08-21 15:01:32.139445+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>34081</t>
+          <t>34750</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026년 하반기 정보보호 전문서비스 기업 지정에 관한 공고</t>
+          <t>｢2026 블록체인 진흥주간｣ 전시부스 참가기업 모집 공고(~9.14)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3742&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3743&amp;page=1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -990,7 +994,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -998,11 +1002,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -1010,44 +1010,44 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-08-13 09:31:24.927741+09:00</t>
+          <t>2026-08-13 17:46:21.938331+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-08-13 09:31:24.927741+09:00</t>
+          <t>2026-08-13 17:46:21.938331+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>34071</t>
+          <t>34081</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>978</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>"예방 넘어 대응·복구까지" 랜섬웨어 전주기 대응 방안 논의한다</t>
+          <t>2026년 하반기 정보보호 전문서비스 기업 지정에 관한 공고</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2626&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3742&amp;page=1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1055,42 +1055,46 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-08-13 09:16:35.989405+09:00</t>
+          <t>2026-08-13 09:31:24.927741+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-08-13 09:16:35.989405+09:00</t>
+          <t>2026-08-13 09:31:24.927741+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>33789</t>
+          <t>34071</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>978</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 21회차 교육생 모집(~9.11)</t>
+          <t>"예방 넘어 대응·복구까지" 랜섬웨어 전주기 대응 방안 논의한다</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3741&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2626&amp;page=1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1100,35 +1104,35 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-08-12 16:01:25.579701+09:00</t>
+          <t>2026-08-13 09:16:35.989405+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-08-12 16:01:25.579701+09:00</t>
+          <t>2026-08-13 09:16:35.989405+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>33749</t>
+          <t>33789</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1138,12 +1142,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026년도 블록체인 유공 포상 계획 공고 안내(~9.21 15:00 마감)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 21회차 교육생 모집(~9.11)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3740&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3741&amp;page=1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1153,12 +1157,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
@@ -1169,44 +1173,44 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-08-12 15:31:25.306307+09:00</t>
+          <t>2026-08-12 16:01:25.579701+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-08-12 15:31:25.306307+09:00</t>
+          <t>2026-08-12 16:01:25.579701+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>31741</t>
+          <t>33749</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026년 블록체인 수요-공급 협의체 (ABLE) 정례세미나 개최 안내(8.13.목)</t>
+          <t>2026년도 블록체인 유공 포상 계획 공고 안내(~9.21 15:00 마감)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3739&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3740&amp;page=1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1214,11 +1218,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -1226,52 +1226,56 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-08-10 11:01:30.246604+09:00</t>
+          <t>2026-08-12 15:31:25.306307+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-08-10 11:01:30.246604+09:00</t>
+          <t>2026-08-12 15:31:25.306307+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>29768</t>
+          <t>31741</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026년 블록체인 신뢰인프라(K-BTF) 활용·확산사업 공모 사전예고</t>
+          <t>2026년 블록체인 수요-공급 협의체 (ABLE) 정례세미나 개최 안내(8.13.목)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3738&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3739&amp;page=1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>13</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -1279,19 +1283,19 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-08-07 17:01:29.954014+09:00</t>
+          <t>2026-08-10 11:01:30.246604+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-08-07 17:01:29.954014+09:00</t>
+          <t>2026-08-10 11:01:30.246604+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>29728</t>
+          <t>29768</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1301,12 +1305,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026년도 블록체인 산업 실태조사 실시 및 협조 안내</t>
+          <t>2026년 블록체인 신뢰인프라(K-BTF) 활용·확산사업 공모 사전예고</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3737&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3738&amp;page=1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1316,7 +1320,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1332,19 +1336,19 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-08-07 16:31:30.938844+09:00</t>
+          <t>2026-08-07 17:01:29.954014+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-08-07 16:31:30.938844+09:00</t>
+          <t>2026-08-07 17:01:29.954014+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>28711</t>
+          <t>29728</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1354,50 +1358,50 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원-나주시, 고교생 개인정보·정보보호 진로 탐색 지원</t>
+          <t>2026년도 블록체인 산업 실태조사 실시 및 협조 안내</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2625&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3737&amp;page=1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-08-06 14:01:34.968573+09:00</t>
+          <t>2026-08-07 16:31:30.938844+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-08-06 14:01:34.968573+09:00</t>
+          <t>2026-08-07 16:31:30.938844+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>27551</t>
+          <t>28711</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1407,22 +1411,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 기업 맞춤형 사이버 위협 알림 서비스 개시</t>
+          <t>한국인터넷진흥원-나주시, 고교생 개인정보·정보보호 진로 탐색 지원</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2624&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2625&amp;page=1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>101</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1438,44 +1442,44 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-08-05 09:46:34.063806+09:00</t>
+          <t>2026-08-06 14:01:34.968573+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-08-05 09:46:34.063806+09:00</t>
+          <t>2026-08-06 14:01:34.968573+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>27511</t>
+          <t>27551</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>975</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 기관장 주도 국민 체감 성과 혁신 체계 가동</t>
+          <t>한국인터넷진흥원, 기업 맞춤형 사이버 위협 알림 서비스 개시</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2623&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2624&amp;page=1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>263</t>
+          <t>101</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1491,34 +1495,34 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-08-05 09:16:33.823896+09:00</t>
+          <t>2026-08-05 09:46:34.063806+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-08-05 09:16:33.823896+09:00</t>
+          <t>2026-08-05 09:46:34.063806+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>27268</t>
+          <t>27511</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>975</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>양자내성암호 국제 표준화 동향 분석</t>
+          <t>한국인터넷진흥원, 기관장 주도 국민 체감 성과 혁신 체계 가동</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3736&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2623&amp;page=1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1528,7 +1532,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>263</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1539,24 +1543,24 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-08-04 16:31:26.502205+09:00</t>
+          <t>2026-08-05 09:16:33.823896+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-08-04 16:31:26.502205+09:00</t>
+          <t>2026-08-05 09:16:33.823896+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>27128</t>
+          <t>27268</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1566,12 +1570,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 20회차 교육생 모집(~9.4)</t>
+          <t>양자내성암호 국제 표준화 동향 분석</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3735&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3736&amp;page=1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1581,12 +1585,12 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
@@ -1597,19 +1601,19 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-08-04 14:46:28.764255+09:00</t>
+          <t>2026-08-04 16:31:26.502205+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-08-04 14:46:28.764255+09:00</t>
+          <t>2026-08-04 16:31:26.502205+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>26211</t>
+          <t>27128</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1619,50 +1623,50 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 암호모듈검증 위한 시험 전문인력 양성</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 20회차 교육생 모집(~9.4)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2622&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3735&amp;page=1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>273</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-08-03 13:31:41.722921+09:00</t>
+          <t>2026-08-04 14:46:28.764255+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-08-03 13:31:41.722921+09:00</t>
+          <t>2026-08-04 14:46:28.764255+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>26188</t>
+          <t>26211</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1672,12 +1676,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026년 8차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(8월 추천) (~8.21(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 암호모듈검증 위한 시험 전문인력 양성</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3734&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2622&amp;page=1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1687,7 +1691,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>273</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1698,24 +1702,24 @@
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-08-03 13:16:30.325331+09:00</t>
+          <t>2026-08-03 13:31:41.722921+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-08-03 13:16:30.325331+09:00</t>
+          <t>2026-08-03 13:31:41.722921+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>25891</t>
+          <t>26188</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1725,12 +1729,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 지역 상생 3대 사업 참여자 모집</t>
+          <t>2026년 8차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(8월 추천) (~8.21(금) 18시까지)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2621&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3734&amp;page=1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1740,7 +1744,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1751,39 +1755,39 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-08-03 09:31:46.854132+09:00</t>
+          <t>2026-08-03 13:16:30.325331+09:00</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-08-03 09:31:46.854132+09:00</t>
+          <t>2026-08-03 13:16:30.325331+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>25864</t>
+          <t>25891</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026년 전남광주통합특별시 소상공인·사회적경제기업 판로 확대 지원기업 선발 안내(~8.14)</t>
+          <t>한국인터넷진흥원, 지역 상생 3대 사업 참여자 모집</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3730&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2621&amp;page=1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1793,7 +1797,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>80</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1801,31 +1805,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-08-03 09:16:35.817723+09:00</t>
+          <t>2026-08-03 09:31:46.854132+09:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-08-03 09:16:35.817723+09:00</t>
+          <t>2026-08-03 09:31:46.854132+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>25863</t>
+          <t>25864</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1835,12 +1835,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026년 전남광주통합특별시 지역문제 해결 프로젝트 공모전 개최 안내(~8.21)</t>
+          <t>2026년 전남광주통합특별시 소상공인·사회적경제기업 판로 확대 지원기업 선발 안내(~8.14)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3731&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3730&amp;page=1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1850,7 +1850,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1882,7 +1882,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>25862</t>
+          <t>25863</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1892,12 +1892,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026년 한국인터넷진흥원 지역공부방 참여 대학생 장학금 지원자 모집 안내(~8.28)</t>
+          <t>2026년 전남광주통합특별시 지역문제 해결 프로젝트 공모전 개최 안내(~8.21)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3732&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3731&amp;page=1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1907,7 +1907,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1939,7 +1939,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>25861</t>
+          <t>25862</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1949,12 +1949,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026년 암호모듈 시험자 양성교육 및 필기시험 안내(8.3~8.21)</t>
+          <t>2026년 한국인터넷진흥원 지역공부방 참여 대학생 장학금 지원자 모집 안내(~8.28)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3733&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3732&amp;page=1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1996,7 +1996,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>23221</t>
+          <t>25861</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2006,22 +2006,22 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026년 블록체인 기업성장허브 입주기업 모집(~8월 27일(목) 16:00까지)</t>
+          <t>2026년 암호모듈 시험자 양성교육 및 필기시험 안내(8.3~8.21)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3729&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3733&amp;page=1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2041,52 +2041,56 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-07-30 17:16:54.540202+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-30 17:16:54.540202+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>22504</t>
+          <t>23221</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 19회차 교육생 모집(~8.28)</t>
+          <t>2026년 블록체인 기업성장허브 입주기업 모집(~8월 27일(목) 16:00까지)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3728&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3729&amp;page=1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -2094,19 +2098,19 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-07-29 18:32:00.075123+09:00</t>
+          <t>2026-07-30 17:16:54.540202+09:00</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-29 18:32:00.075123+09:00</t>
+          <t>2026-07-30 17:16:54.540202+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>22464</t>
+          <t>22504</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2116,12 +2120,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026년 연계정보 이용기관 안전조치 실태점검 2차 설명회 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 19회차 교육생 모집(~8.28)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3727&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3728&amp;page=1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2131,7 +2135,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2147,19 +2151,19 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-07-29 18:01:59.875668+09:00</t>
+          <t>2026-07-29 18:32:00.075123+09:00</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-29 18:01:59.875668+09:00</t>
+          <t>2026-07-29 18:32:00.075123+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>20771</t>
+          <t>22464</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2169,50 +2173,50 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
+          <t>2026년 연계정보 이용기관 안전조치 실태점검 2차 설명회 개최</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3727&amp;page=1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>20191</t>
+          <t>20771</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2222,12 +2226,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
+          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2237,7 +2241,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>287</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2253,34 +2257,34 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>20061</t>
+          <t>20191</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
+          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2290,7 +2294,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>246</t>
+          <t>287</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2298,64 +2302,64 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>16785</t>
+          <t>20061</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>1496</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
+          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>246</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -2363,34 +2367,34 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>16784</t>
+          <t>16785</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>1497</t>
+          <t>1496</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2400,7 +2404,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>236</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2428,22 +2432,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>16781</t>
+          <t>16784</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1497</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2453,7 +2457,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>260</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2461,11 +2465,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -2485,22 +2485,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>16691</t>
+          <t>16781</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2510,35 +2510,39 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>278</t>
+          <t>242</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>16464</t>
+          <t>16691</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2548,12 +2552,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
+          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2563,35 +2567,35 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>278</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>16051</t>
+          <t>16464</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2601,12 +2605,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
+          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2616,35 +2620,35 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>14611</t>
+          <t>16051</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2654,22 +2658,22 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
+          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>233</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2685,19 +2689,19 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>14431</t>
+          <t>14611</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2707,12 +2711,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2722,7 +2726,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2738,34 +2742,34 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>14431</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2775,7 +2779,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2783,56 +2787,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>14444</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>1493</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2840,7 +2840,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I45" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -2848,34 +2852,34 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>11331</t>
+          <t>14444</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1493</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2885,7 +2889,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2896,96 +2900,92 @@
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>10981</t>
+          <t>11331</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
+          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>10943</t>
+          <t>10981</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
+          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2995,7 +2995,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3003,7 +3003,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I48" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -3011,19 +3015,19 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>10663</t>
+          <t>10943</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -3033,12 +3037,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
+          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -3048,12 +3052,12 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H49" t="inlineStr"/>
@@ -3064,19 +3068,19 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>9805</t>
+          <t>10663</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3086,22 +3090,22 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
+          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3117,19 +3121,19 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>9691</t>
+          <t>9805</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3139,12 +3143,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
+          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -3154,7 +3158,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3165,96 +3169,92 @@
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>9321</t>
+          <t>9691</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
+          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>8871</t>
+          <t>9321</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
+          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -3264,35 +3264,39 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>6685</t>
+          <t>8871</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3302,22 +3306,22 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
+          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -3328,24 +3332,24 @@
       <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>6571</t>
+          <t>6685</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3355,12 +3359,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
+          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -3370,7 +3374,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -3381,24 +3385,24 @@
       <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>5591</t>
+          <t>6571</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3408,22 +3412,22 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
+          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3439,44 +3443,44 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>5591</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
+          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3492,44 +3496,44 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>4762</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>961</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>AI 보안 위협 대응 매뉴얼</t>
+          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -3537,31 +3541,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>4761</t>
+          <t>4762</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3571,12 +3571,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>AI 보안 레드티밍 가이드</t>
+          <t>AI 보안 위협 대응 매뉴얼</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -3586,7 +3586,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -3618,22 +3618,22 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>4761</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
+          <t>AI 보안 레드티밍 가이드</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3643,7 +3643,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -3651,27 +3651,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3681,12 +3685,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
+          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3696,113 +3700,113 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>191</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>3867</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
+          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4111</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>959</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3810,31 +3814,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3844,12 +3844,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
+          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3859,7 +3859,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3891,32 +3891,32 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>1477</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
+          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3924,7 +3924,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr"/>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I65" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -3944,22 +3948,22 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>1477</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
+          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3969,7 +3973,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>386</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3997,22 +4001,22 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
+          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -4022,19 +4026,15 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>362</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -4054,7 +4054,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -4064,12 +4064,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2026년 IoT 보안인증 교육과정 안내</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -4079,7 +4079,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>522</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -4111,40 +4111,44 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
+          <t>2026년 IoT 보안인증 교육과정 안내</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>652</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H69" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I69" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -4164,22 +4168,22 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
+          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -4189,7 +4193,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>818</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -4197,11 +4201,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H70" t="inlineStr"/>
       <c r="I70" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -4221,32 +4221,32 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
+          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>2264</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -4254,7 +4254,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I71" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -4262,34 +4266,34 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>958</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -4299,7 +4303,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>76426</t>
+          <t>2264</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -4310,49 +4314,49 @@
       <c r="H72" t="inlineStr"/>
       <c r="I72" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>956</t>
+          <t>958</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
+          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>55906</t>
+          <t>76426</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -4380,22 +4384,22 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>957</t>
+          <t>956</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
+          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -4405,7 +4409,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>55329</t>
+          <t>55906</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -4433,32 +4437,32 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>955</t>
+          <t>957</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
+          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>34467</t>
+          <t>55329</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -4486,22 +4490,22 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>955</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
+          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -4511,39 +4515,35 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>2945</t>
+          <t>34467</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr"/>
       <c r="I76" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -4553,27 +4553,27 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>5048</t>
+          <t>2945</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -4600,32 +4600,32 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>954</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>145255</t>
+          <t>5048</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -4633,52 +4633,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr"/>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>954</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>26576</t>
+          <t>145255</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -4706,32 +4710,32 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>952</t>
+          <t>953</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
+          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>34290</t>
+          <t>26576</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -4759,32 +4763,32 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>951</t>
+          <t>952</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>184573</t>
+          <t>34290</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -4812,32 +4816,32 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>14403</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>951</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>6587</t>
+          <t>184573</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -4845,46 +4849,42 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H82" t="inlineStr"/>
       <c r="I82" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>14403</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -4894,7 +4894,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>51749</t>
+          <t>6587</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -4902,52 +4902,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>949</t>
+          <t>950</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>78439</t>
+          <t>51749</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -4975,55 +4979,108 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>949</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>78439</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
           <t>38805</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr">
+      <c r="B86" t="inlineStr">
         <is>
           <t>공지</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
+      <c r="C86" t="inlineStr">
         <is>
           <t>[공유] 지능형 CCTV 성능시험 재개 안내 공지</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr">
+      <c r="D86" t="inlineStr">
         <is>
           <t>https://www.kisa.or.kr/401/form?postSeq=3677&amp;page=1</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
+      <c r="E86" t="inlineStr">
         <is>
           <t>2026-06-02</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr">
+      <c r="F86" t="inlineStr">
         <is>
           <t>6525</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr">
+      <c r="G86" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr">
+      <c r="H86" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>공지사항</t>
-        </is>
-      </c>
-      <c r="J85" t="inlineStr">
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>공지사항</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
         <is>
           <t>2026-08-18 17:16:37.364015+09:00</t>
         </is>
       </c>
-      <c r="K85" t="inlineStr">
+      <c r="K86" t="inlineStr">
         <is>
           <t>2026-08-18 17:16:37.364015+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-09-01 10:20:02 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/kisa.xlsx
+++ b/docs/snapshot/downloads/kisa.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K90"/>
+  <dimension ref="A1:K91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,7 +476,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>49631</t>
+          <t>49669</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -486,12 +486,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>물리보안 시스템 간 연동 장벽 낮춘다</t>
+          <t>「2026 위치정보 맞춤형 컨설팅 참여기업 모집」</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2632&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3752&amp;page=1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -501,103 +501,103 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>13</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-01 09:01:45.980040+09:00</t>
+          <t>2026-09-01 09:31:38.715793+09:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-09-01 09:01:45.980040+09:00</t>
+          <t>2026-09-01 09:31:38.715793+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>49589</t>
+          <t>49631</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1517</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 23회차 교육생 모집(~9.18)</t>
+          <t>물리보안 시스템 간 연동 장벽 낮춘다</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3751&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2632&amp;page=1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>174</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-01 08:31:37.253592+09:00</t>
+          <t>2026-09-01 09:01:45.980040+09:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-09-01 08:31:37.253592+09:00</t>
+          <t>2026-09-01 09:01:45.980040+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>48831</t>
+          <t>49589</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1517</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>생성형 인공지능(AI) 기반 실전형 모의해킹 대회 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 23회차 교육생 모집(~9.18)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2630&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3751&amp;page=1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -607,35 +607,35 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>174</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-08-31 09:16:38.866405+09:00</t>
+          <t>2026-09-01 08:31:37.253592+09:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-08-31 09:16:38.866405+09:00</t>
+          <t>2026-09-01 08:31:37.253592+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>46011</t>
+          <t>48831</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -645,22 +645,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>자동차 노리는 사이버 위협, 한국인터넷진흥원-한국교통안전공단이 함께 대응한다</t>
+          <t>생성형 인공지능(AI) 기반 실전형 모의해킹 대회 개최</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2628&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2630&amp;page=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -676,34 +676,34 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-08-27 15:01:41.552844+09:00</t>
+          <t>2026-08-31 09:16:38.866405+09:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-08-27 15:01:41.552844+09:00</t>
+          <t>2026-08-31 09:16:38.866405+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>45681</t>
+          <t>46011</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>싱가포르 현지 진출 지원 국내 블록체인 기업 모집(~9.16(수) 14시)</t>
+          <t>자동차 노리는 사이버 위협, 한국인터넷진흥원-한국교통안전공단이 함께 대응한다</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3750&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2628&amp;page=1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -721,56 +721,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-08-27 11:01:31.314899+09:00</t>
+          <t>2026-08-27 15:01:41.552844+09:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-08-27 11:01:31.314899+09:00</t>
+          <t>2026-08-27 15:01:41.552844+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>45191</t>
+          <t>45681</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 아·태 지역 사이버공격 대응 공동 훈련 실시</t>
+          <t>싱가포르 현지 진출 지원 국내 블록체인 기업 모집(~9.16(수) 14시)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2629&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3750&amp;page=1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -778,42 +774,46 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-08-26 15:01:47.261933+09:00</t>
+          <t>2026-08-27 11:01:31.314899+09:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-08-26 15:01:47.261933+09:00</t>
+          <t>2026-08-27 11:01:31.314899+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>44741</t>
+          <t>45191</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>[3차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~9/16)</t>
+          <t>한국인터넷진흥원, 아·태 지역 사이버공격 대응 공동 훈련 실시</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3749&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2629&amp;page=1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -823,7 +823,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -831,56 +831,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-08-26 09:31:36.427758+09:00</t>
+          <t>2026-08-26 15:01:47.261933+09:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-08-26 09:31:36.427758+09:00</t>
+          <t>2026-08-26 15:01:47.261933+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>44448</t>
+          <t>44741</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 공고</t>
+          <t>[3차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~9/16)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3748&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3749&amp;page=1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -888,7 +884,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -896,19 +896,19 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-08-25 16:01:39.626193+09:00</t>
+          <t>2026-08-26 09:31:36.427758+09:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-08-25 16:01:39.626193+09:00</t>
+          <t>2026-08-26 09:31:36.427758+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>43767</t>
+          <t>44448</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -918,27 +918,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 21회차 교육생 모집(~9.12)</t>
+          <t>정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 공고</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3747&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3748&amp;page=1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -949,19 +949,19 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-08-24 17:46:42.254577+09:00</t>
+          <t>2026-08-25 16:01:39.626193+09:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-08-24 17:46:42.254577+09:00</t>
+          <t>2026-08-25 16:01:39.626193+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>43311</t>
+          <t>43767</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -971,12 +971,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>양자내성암호 전환, 어떻게 준비해야 할까?</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 21회차 교육생 모집(~9.12)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2627&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3747&amp;page=1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -986,50 +986,50 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-08-24 12:01:45.511381+09:00</t>
+          <t>2026-08-24 17:46:42.254577+09:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-08-24 12:01:45.511381+09:00</t>
+          <t>2026-08-24 17:46:42.254577+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>43301</t>
+          <t>43311</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 실무과정 교육생 모집(8.24~)</t>
+          <t>양자내성암호 전환, 어떻게 준비해야 할까?</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3746&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2627&amp;page=1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1047,31 +1047,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-08-24 12:01:36.271108+09:00</t>
+          <t>2026-08-24 12:01:45.511381+09:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-08-24 12:01:36.271108+09:00</t>
+          <t>2026-08-24 12:01:45.511381+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>41161</t>
+          <t>43301</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1081,27 +1077,27 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>「블록체인 기업 맞춤형 보안 고도화 지원」 기업 모집(~8/31)</t>
+          <t>양자내성암호 전문교육 PQC 실무과정 교육생 모집(8.24~)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3745&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3746&amp;page=1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1116,34 +1112,34 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-08-21 16:01:38.087170+09:00</t>
+          <t>2026-08-24 12:01:36.271108+09:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-08-21 16:01:38.087170+09:00</t>
+          <t>2026-08-24 12:01:36.271108+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>41086</t>
+          <t>41161</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026년도 인터넷거버넌스 민간전문가 APrIGF 및 IGF 참석자 모집</t>
+          <t>「블록체인 기업 맞춤형 보안 고도화 지원」 기업 모집(~8/31)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3744&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3745&amp;page=1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1153,15 +1149,19 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -1169,19 +1169,19 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-08-21 15:01:32.139445+09:00</t>
+          <t>2026-08-21 16:01:38.087170+09:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-08-21 15:01:32.139445+09:00</t>
+          <t>2026-08-21 16:01:38.087170+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>34750</t>
+          <t>41086</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1191,22 +1191,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>｢2026 블록체인 진흥주간｣ 전시부스 참가기업 모집 공고(~9.14)</t>
+          <t>2026년도 인터넷거버넌스 민간전문가 APrIGF 및 IGF 참석자 모집</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3743&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3744&amp;page=1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>59</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1222,34 +1222,34 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-08-13 17:46:21.938331+09:00</t>
+          <t>2026-08-21 15:01:32.139445+09:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-08-13 17:46:21.938331+09:00</t>
+          <t>2026-08-21 15:01:32.139445+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>34081</t>
+          <t>34750</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026년 하반기 정보보호 전문서비스 기업 지정에 관한 공고</t>
+          <t>｢2026 블록체인 진흥주간｣ 전시부스 참가기업 모집 공고(~9.14)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3742&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3743&amp;page=1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1267,11 +1267,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -1279,44 +1275,44 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-08-13 09:31:24.927741+09:00</t>
+          <t>2026-08-13 17:46:21.938331+09:00</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-08-13 09:31:24.927741+09:00</t>
+          <t>2026-08-13 17:46:21.938331+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>34071</t>
+          <t>34081</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>978</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>"예방 넘어 대응·복구까지" 랜섬웨어 전주기 대응 방안 논의한다</t>
+          <t>2026년 하반기 정보보호 전문서비스 기업 지정에 관한 공고</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2626&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3742&amp;page=1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1324,42 +1320,46 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-08-13 09:16:35.989405+09:00</t>
+          <t>2026-08-13 09:31:24.927741+09:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-08-13 09:16:35.989405+09:00</t>
+          <t>2026-08-13 09:31:24.927741+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>33789</t>
+          <t>34071</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>978</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 21회차 교육생 모집(~9.11)</t>
+          <t>"예방 넘어 대응·복구까지" 랜섬웨어 전주기 대응 방안 논의한다</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3741&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2626&amp;page=1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1369,35 +1369,35 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-08-12 16:01:25.579701+09:00</t>
+          <t>2026-08-13 09:16:35.989405+09:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-08-12 16:01:25.579701+09:00</t>
+          <t>2026-08-13 09:16:35.989405+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>33749</t>
+          <t>33789</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1407,12 +1407,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026년도 블록체인 유공 포상 계획 공고 안내(~9.21 15:00 마감)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 21회차 교육생 모집(~9.11)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3740&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3741&amp;page=1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1422,12 +1422,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -1438,44 +1438,44 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-08-12 15:31:25.306307+09:00</t>
+          <t>2026-08-12 16:01:25.579701+09:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-08-12 15:31:25.306307+09:00</t>
+          <t>2026-08-12 16:01:25.579701+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>31741</t>
+          <t>33749</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026년 블록체인 수요-공급 협의체 (ABLE) 정례세미나 개최 안내(8.13.목)</t>
+          <t>2026년도 블록체인 유공 포상 계획 공고 안내(~9.21 15:00 마감)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3739&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3740&amp;page=1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1483,11 +1483,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -1495,52 +1491,56 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-08-10 11:01:30.246604+09:00</t>
+          <t>2026-08-12 15:31:25.306307+09:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-08-10 11:01:30.246604+09:00</t>
+          <t>2026-08-12 15:31:25.306307+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>29768</t>
+          <t>31741</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026년 블록체인 신뢰인프라(K-BTF) 활용·확산사업 공모 사전예고</t>
+          <t>2026년 블록체인 수요-공급 협의체 (ABLE) 정례세미나 개최 안내(8.13.목)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3738&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3739&amp;page=1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>13</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -1548,19 +1548,19 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-08-07 17:01:29.954014+09:00</t>
+          <t>2026-08-10 11:01:30.246604+09:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-08-07 17:01:29.954014+09:00</t>
+          <t>2026-08-10 11:01:30.246604+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>29728</t>
+          <t>29768</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1570,12 +1570,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026년도 블록체인 산업 실태조사 실시 및 협조 안내</t>
+          <t>2026년 블록체인 신뢰인프라(K-BTF) 활용·확산사업 공모 사전예고</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3737&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3738&amp;page=1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1585,7 +1585,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1601,19 +1601,19 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-08-07 16:31:30.938844+09:00</t>
+          <t>2026-08-07 17:01:29.954014+09:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-08-07 16:31:30.938844+09:00</t>
+          <t>2026-08-07 17:01:29.954014+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>28711</t>
+          <t>29728</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1623,50 +1623,50 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원-나주시, 고교생 개인정보·정보보호 진로 탐색 지원</t>
+          <t>2026년도 블록체인 산업 실태조사 실시 및 협조 안내</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2625&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3737&amp;page=1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-08-06 14:01:34.968573+09:00</t>
+          <t>2026-08-07 16:31:30.938844+09:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-08-06 14:01:34.968573+09:00</t>
+          <t>2026-08-07 16:31:30.938844+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>27551</t>
+          <t>28711</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1676,22 +1676,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 기업 맞춤형 사이버 위협 알림 서비스 개시</t>
+          <t>한국인터넷진흥원-나주시, 고교생 개인정보·정보보호 진로 탐색 지원</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2624&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2625&amp;page=1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>101</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1707,44 +1707,44 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-08-05 09:46:34.063806+09:00</t>
+          <t>2026-08-06 14:01:34.968573+09:00</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-08-05 09:46:34.063806+09:00</t>
+          <t>2026-08-06 14:01:34.968573+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>27511</t>
+          <t>27551</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>975</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 기관장 주도 국민 체감 성과 혁신 체계 가동</t>
+          <t>한국인터넷진흥원, 기업 맞춤형 사이버 위협 알림 서비스 개시</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2623&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2624&amp;page=1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>263</t>
+          <t>101</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1760,34 +1760,34 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-08-05 09:16:33.823896+09:00</t>
+          <t>2026-08-05 09:46:34.063806+09:00</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-08-05 09:16:33.823896+09:00</t>
+          <t>2026-08-05 09:46:34.063806+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>27268</t>
+          <t>27511</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>975</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>양자내성암호 국제 표준화 동향 분석</t>
+          <t>한국인터넷진흥원, 기관장 주도 국민 체감 성과 혁신 체계 가동</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3736&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2623&amp;page=1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>263</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1808,24 +1808,24 @@
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-08-04 16:31:26.502205+09:00</t>
+          <t>2026-08-05 09:16:33.823896+09:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-08-04 16:31:26.502205+09:00</t>
+          <t>2026-08-05 09:16:33.823896+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>27128</t>
+          <t>27268</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1835,12 +1835,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 20회차 교육생 모집(~9.4)</t>
+          <t>양자내성암호 국제 표준화 동향 분석</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3735&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3736&amp;page=1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1850,12 +1850,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
@@ -1866,19 +1866,19 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-08-04 14:46:28.764255+09:00</t>
+          <t>2026-08-04 16:31:26.502205+09:00</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-08-04 14:46:28.764255+09:00</t>
+          <t>2026-08-04 16:31:26.502205+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>26211</t>
+          <t>27128</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1888,50 +1888,50 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 암호모듈검증 위한 시험 전문인력 양성</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 20회차 교육생 모집(~9.4)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2622&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3735&amp;page=1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>273</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-08-03 13:31:41.722921+09:00</t>
+          <t>2026-08-04 14:46:28.764255+09:00</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-08-03 13:31:41.722921+09:00</t>
+          <t>2026-08-04 14:46:28.764255+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>26188</t>
+          <t>26211</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1941,12 +1941,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026년 8차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(8월 추천) (~8.21(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 암호모듈검증 위한 시험 전문인력 양성</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3734&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2622&amp;page=1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>273</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1967,24 +1967,24 @@
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-08-03 13:16:30.325331+09:00</t>
+          <t>2026-08-03 13:31:41.722921+09:00</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-08-03 13:16:30.325331+09:00</t>
+          <t>2026-08-03 13:31:41.722921+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>25891</t>
+          <t>26188</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1994,12 +1994,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 지역 상생 3대 사업 참여자 모집</t>
+          <t>2026년 8차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(8월 추천) (~8.21(금) 18시까지)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2621&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3734&amp;page=1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2009,7 +2009,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2020,39 +2020,39 @@
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-08-03 09:31:46.854132+09:00</t>
+          <t>2026-08-03 13:16:30.325331+09:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-08-03 09:31:46.854132+09:00</t>
+          <t>2026-08-03 13:16:30.325331+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>25864</t>
+          <t>25891</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026년 전남광주통합특별시 소상공인·사회적경제기업 판로 확대 지원기업 선발 안내(~8.14)</t>
+          <t>한국인터넷진흥원, 지역 상생 3대 사업 참여자 모집</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3730&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2621&amp;page=1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2062,7 +2062,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>80</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2070,31 +2070,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-08-03 09:16:35.817723+09:00</t>
+          <t>2026-08-03 09:31:46.854132+09:00</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-08-03 09:16:35.817723+09:00</t>
+          <t>2026-08-03 09:31:46.854132+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>25863</t>
+          <t>25864</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2104,12 +2100,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026년 전남광주통합특별시 지역문제 해결 프로젝트 공모전 개최 안내(~8.21)</t>
+          <t>2026년 전남광주통합특별시 소상공인·사회적경제기업 판로 확대 지원기업 선발 안내(~8.14)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3731&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3730&amp;page=1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2119,7 +2115,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2151,7 +2147,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>25862</t>
+          <t>25863</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2161,12 +2157,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026년 한국인터넷진흥원 지역공부방 참여 대학생 장학금 지원자 모집 안내(~8.28)</t>
+          <t>2026년 전남광주통합특별시 지역문제 해결 프로젝트 공모전 개최 안내(~8.21)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3732&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3731&amp;page=1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2176,7 +2172,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2208,7 +2204,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>25861</t>
+          <t>25862</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2218,12 +2214,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026년 암호모듈 시험자 양성교육 및 필기시험 안내(8.3~8.21)</t>
+          <t>2026년 한국인터넷진흥원 지역공부방 참여 대학생 장학금 지원자 모집 안내(~8.28)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3733&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3732&amp;page=1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2233,7 +2229,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2265,7 +2261,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>23221</t>
+          <t>25861</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2275,22 +2271,22 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026년 블록체인 기업성장허브 입주기업 모집(~8월 27일(목) 16:00까지)</t>
+          <t>2026년 암호모듈 시험자 양성교육 및 필기시험 안내(8.3~8.21)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3729&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3733&amp;page=1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2310,52 +2306,56 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-07-30 17:16:54.540202+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-07-30 17:16:54.540202+09:00</t>
+          <t>2026-08-03 09:16:35.817723+09:00</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>22504</t>
+          <t>23221</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 19회차 교육생 모집(~8.28)</t>
+          <t>2026년 블록체인 기업성장허브 입주기업 모집(~8월 27일(목) 16:00까지)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3728&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3729&amp;page=1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -2363,19 +2363,19 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-07-29 18:32:00.075123+09:00</t>
+          <t>2026-07-30 17:16:54.540202+09:00</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-07-29 18:32:00.075123+09:00</t>
+          <t>2026-07-30 17:16:54.540202+09:00</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>22464</t>
+          <t>22504</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2385,12 +2385,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026년 연계정보 이용기관 안전조치 실태점검 2차 설명회 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 19회차 교육생 모집(~8.28)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3727&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3728&amp;page=1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2400,7 +2400,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2416,19 +2416,19 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-07-29 18:01:59.875668+09:00</t>
+          <t>2026-07-29 18:32:00.075123+09:00</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-07-29 18:01:59.875668+09:00</t>
+          <t>2026-07-29 18:32:00.075123+09:00</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>20771</t>
+          <t>22464</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2438,50 +2438,50 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
+          <t>2026년 연계정보 이용기관 안전조치 실태점검 2차 설명회 개최</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3727&amp;page=1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-07-27 17:17:05.702970+09:00</t>
+          <t>2026-07-29 18:01:59.875668+09:00</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>20191</t>
+          <t>20771</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2491,12 +2491,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
+          <t>한국인터넷진흥원, 성평등가족부와 불법·유해 정보 유통 대응 맞손</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2620&amp;page=1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2506,7 +2506,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>287</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2522,34 +2522,34 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-07-27 10:02:05.338547+09:00</t>
+          <t>2026-07-27 17:17:05.702970+09:00</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>20061</t>
+          <t>20191</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
+          <t>아피가(APIGA) 향후 10년 설계한다…전담 추진단(TF) 출범</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2619&amp;page=1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2559,7 +2559,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>246</t>
+          <t>287</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2567,64 +2567,64 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-07-27 08:31:55.019743+09:00</t>
+          <t>2026-07-27 10:02:05.338547+09:00</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>16785</t>
+          <t>20061</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>1496</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
+          <t>2026년 정보보호제품 성능평가자 양성교육 신청·접수 안내(1차, BreakingPoint)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3726&amp;page=1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>246</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I41" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -2632,34 +2632,34 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-07-23 08:31:55.372982+09:00</t>
+          <t>2026-07-27 08:31:55.019743+09:00</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>16784</t>
+          <t>16785</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>1497</t>
+          <t>1496</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 17회차 교육생 모집(~8.7)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3724&amp;page=1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2669,7 +2669,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>236</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2697,22 +2697,22 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>16781</t>
+          <t>16784</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1497</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 18회차 교육생 모집(~8.21)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3725&amp;page=1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2722,7 +2722,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>260</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2730,11 +2730,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -2754,22 +2750,22 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>16691</t>
+          <t>16781</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 16회차 교육생 모집(~7.31)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3723&amp;page=1</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2779,35 +2775,39 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>278</t>
+          <t>242</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-07-22 17:32:01.526863+09:00</t>
+          <t>2026-07-23 08:31:55.372982+09:00</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>16464</t>
+          <t>16691</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2817,12 +2817,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
+          <t>'블록체인 기반 예금토큰 결제 인프라 확산' 사업 발대식 개최</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2618&amp;page=1</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2832,35 +2832,35 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>278</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-07-22 14:46:48.687665+09:00</t>
+          <t>2026-07-22 17:32:01.526863+09:00</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>16051</t>
+          <t>16464</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2870,12 +2870,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
+          <t>[홍보] 정보보호특성화대학 대상 사이버전문사관 제3기 후보생 모집·선발 안내</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3722&amp;page=1</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2885,35 +2885,35 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>2026-07-22 09:31:50.671841+09:00</t>
+          <t>2026-07-22 14:46:48.687665+09:00</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>14611</t>
+          <t>16051</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2923,22 +2923,22 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
+          <t>한국인터넷진흥원, 보안 인재·글로벌 전문가 교류의 장 열어</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2617&amp;page=1</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>233</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2954,19 +2954,19 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>2026-07-20 12:01:44.402603+09:00</t>
+          <t>2026-07-22 09:31:50.671841+09:00</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>14431</t>
+          <t>14611</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2976,12 +2976,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>아태지역 15개국 청년, 인터넷거버넌스 미래 함께 그린다</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2616&amp;page=1</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2991,7 +2991,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3007,34 +3007,34 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:51.916450+09:00</t>
+          <t>2026-07-20 12:01:44.402603+09:00</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>14421</t>
+          <t>14431</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2615&amp;page=1</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -3044,7 +3044,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -3052,56 +3052,52 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>2026-07-20 09:46:42.059527+09:00</t>
+          <t>2026-07-20 09:46:51.916450+09:00</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>14444</t>
+          <t>14421</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>1493</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
+          <t>[2차모집]2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3721&amp;page=1</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3109,7 +3105,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I50" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -3117,34 +3117,34 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>2026-07-20 10:01:38.608709+09:00</t>
+          <t>2026-07-20 09:46:42.059527+09:00</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>11331</t>
+          <t>14444</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>1493</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
+          <t>2026년도 개인정보 이노베이션 존 운영기관 지정 공모</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3720&amp;page=1</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -3154,7 +3154,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3165,96 +3165,92 @@
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>2026-07-16 12:01:52.363213+09:00</t>
+          <t>2026-07-20 10:01:38.608709+09:00</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>10981</t>
+          <t>11331</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
+          <t>건설 현장 특화 폐쇄회로 텔레비전(CCTV)으로 안전 지킨다</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2614&amp;page=1</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>2026-07-15 18:01:48.663614+09:00</t>
+          <t>2026-07-16 12:01:52.363213+09:00</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>10943</t>
+          <t>10981</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
+          <t>AI 기반 소스코드 취약점 점검 서비스 안내</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3719&amp;page=1</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -3264,7 +3260,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3272,7 +3268,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I53" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -3280,19 +3280,19 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>2026-07-15 17:31:36.060314+09:00</t>
+          <t>2026-07-15 18:01:48.663614+09:00</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>10663</t>
+          <t>10943</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3302,12 +3302,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
+          <t>일상, 생활, 산업 현장 등에서 활용 가능한 위치정보 기반 안전 솔루션 모집공고</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3718&amp;page=1</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -3317,12 +3317,12 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H54" t="inlineStr"/>
@@ -3333,19 +3333,19 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>2026-07-15 14:01:31.783249+09:00</t>
+          <t>2026-07-15 17:31:36.060314+09:00</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>9805</t>
+          <t>10663</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3355,22 +3355,22 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
+          <t>[공지] 2026년 가명정보 전문인력 양성교육 교육생 모집 및 일정 안내</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3717&amp;page=1</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -3386,19 +3386,19 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>2026-07-14 13:31:36.337069+09:00</t>
+          <t>2026-07-15 14:01:31.783249+09:00</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>9691</t>
+          <t>9805</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3408,12 +3408,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
+          <t>제21회 대한민국 인터넷대상 시상계획 공고</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3716&amp;page=1</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3434,96 +3434,92 @@
       <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>2026-07-14 12:01:56.704390+09:00</t>
+          <t>2026-07-14 13:31:36.337069+09:00</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>9321</t>
+          <t>9691</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
+          <t>대한민국 국가도메인 등록 건수 반등…110만 건대 회복</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2613&amp;page=1</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>2026-07-13 17:46:38.182861+09:00</t>
+          <t>2026-07-14 12:01:56.704390+09:00</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>8871</t>
+          <t>9321</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
+          <t>2026년 팀 시큐리티 코리아 기술세미나 개최 안내(7/22, 서울 로카우스 호텔)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3715&amp;page=1</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -3533,35 +3529,39 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>2026-07-13 12:01:38.210091+09:00</t>
+          <t>2026-07-13 17:46:38.182861+09:00</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>6685</t>
+          <t>8871</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3571,22 +3571,22 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
+          <t>국민 안전 높일 제품·서비스 발굴한다…‘국민안전 위치기반서비스(LBS) 솔루션 대상’ 개최</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2612&amp;page=1</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -3597,24 +3597,24 @@
       <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>2026-07-10 15:31:41.134348+09:00</t>
+          <t>2026-07-13 12:01:38.210091+09:00</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>6571</t>
+          <t>6685</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3624,12 +3624,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
+          <t>공급망 보안 모델 구축 지원사업 회계감사</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3714&amp;page=1</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3639,7 +3639,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -3650,24 +3650,24 @@
       <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>2026-07-10 14:01:48.566995+09:00</t>
+          <t>2026-07-10 15:31:41.134348+09:00</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>5591</t>
+          <t>6571</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3677,22 +3677,22 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
+          <t>“설계에서 실천으로” 기업 공급망 보안 역량 높인다</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2611&amp;page=1</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3708,44 +3708,44 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>2026-07-09 12:01:43.992717+09:00</t>
+          <t>2026-07-10 14:01:48.566995+09:00</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>5591</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
+          <t>한국인터넷진흥원, 부산대 법전원과 인공지능·정보통신기술(ICT) 분쟁 해결 전문인력 양성</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2610&amp;page=1</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -3761,44 +3761,44 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>2026-07-09 09:16:53.071276+09:00</t>
+          <t>2026-07-09 12:01:43.992717+09:00</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>4762</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>961</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>AI 보안 위협 대응 매뉴얼</t>
+          <t>한국인터넷진흥원, 세계은행과 제11회 글로벌 사이버보안 협력 네트워크(CAMP) 연례 회의 개최</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2609&amp;page=1</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3806,31 +3806,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>2026-07-08 12:01:32.847380+09:00</t>
+          <t>2026-07-09 09:16:53.071276+09:00</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>4761</t>
+          <t>4762</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3840,12 +3836,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>AI 보안 레드티밍 가이드</t>
+          <t>AI 보안 위협 대응 매뉴얼</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3712&amp;page=1</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3855,7 +3851,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3887,22 +3883,22 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>4761</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
+          <t>AI 보안 레드티밍 가이드</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3713&amp;page=1</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3912,7 +3908,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3920,27 +3916,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr"/>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>2026-07-07 15:46:43.251266+09:00</t>
+          <t>2026-07-08 12:01:32.847380+09:00</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3950,12 +3950,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
+          <t>“국민 눈높이로 블록체인 서비스 살핀다” 2026년 블록체인 누리단 활동 시작</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2608&amp;page=1</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3965,113 +3965,113 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>191</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>2026-07-07 11:01:32.170051+09:00</t>
+          <t>2026-07-07 15:46:43.251266+09:00</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>3867</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
+          <t>2026년 상반기 침해사고 정보공유 세미나 개최(7/22, 한국과학기술회관)</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3711&amp;page=1</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>2026-07-07 14:01:43.293075+09:00</t>
+          <t>2026-07-07 11:01:32.170051+09:00</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4111</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>959</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
+          <t>한국인터넷진흥원, 엘지유플러스와 음성스팸 대응 협력 강화</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2607&amp;page=1</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -4079,31 +4079,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H68" t="inlineStr"/>
       <c r="I68" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-07 14:01:43.293075+09:00</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -4113,12 +4109,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
+          <t>2026년 7차 정보보호 인증제품 조달청 벤처나라 추천 희망기업 모집 공고(7월 추천) (~7.24(금) 18시까지)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3709&amp;page=1</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -4128,7 +4124,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>243</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -4160,32 +4156,32 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>1477</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
+          <t>2026년 '생성형 AI기반 침해대응체계 도입 및 구축' 사업 설명회(7.10, 판교 정보보호클러스터) 안내</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3710&amp;page=1</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -4193,7 +4189,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr"/>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I70" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -4213,22 +4213,22 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>1477</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
+          <t>국경 간 개인정보 보호 규칙 인증(CBPR) 심사기관 지정 공고</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3707&amp;page=1</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -4238,7 +4238,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>386</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -4266,22 +4266,22 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
+          <t>[접수중] 가명정보 활용 지원사업 성과공유 및 사업설명회 안내</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3708&amp;page=1</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -4291,19 +4291,15 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>362</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr"/>
       <c r="I72" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -4323,7 +4319,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -4333,12 +4329,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2026년 IoT 보안인증 교육과정 안내</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 15회차 교육생 모집(~7.24)</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3705&amp;page=1</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -4348,7 +4344,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>652</t>
+          <t>522</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -4380,40 +4376,44 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
+          <t>2026년 IoT 보안인증 교육과정 안내</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3706&amp;page=1</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>652</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H74" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I74" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -4433,22 +4433,22 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
+          <t>2026년도 우수 정보보호 기술 등 지정 공고</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3704&amp;page=1</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -4458,7 +4458,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>818</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -4466,11 +4466,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H75" t="inlineStr"/>
       <c r="I75" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -4490,32 +4486,32 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>1476</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
+          <t>양자내성암호 전문교육 PQC 개발·전환과정 교육생 모집(6.30~)</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3703&amp;page=1</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>2264</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -4523,7 +4519,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr"/>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I76" t="inlineStr">
         <is>
           <t>공지사항</t>
@@ -4531,34 +4531,34 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>2026-07-04 08:31:28.404468+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>958</t>
+          <t>1476</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
+          <t>2026 개인정보 보호·활용 기술 대상 모집 공고(~7.31(금))</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3702&amp;page=1</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -4568,7 +4568,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>76426</t>
+          <t>2264</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -4579,49 +4579,49 @@
       <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-04 08:31:28.404468+09:00</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>956</t>
+          <t>958</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
+          <t>안전한 개인정보 활용을 위한 연구개발 본격 착수</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2605&amp;page=1</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>55906</t>
+          <t>76426</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -4649,22 +4649,22 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>957</t>
+          <t>956</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
+          <t>한국인터넷진흥원, 협력업체 상생·동반성장 간담회 개최</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2604&amp;page=1</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -4674,7 +4674,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>55329</t>
+          <t>55906</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -4702,32 +4702,32 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>955</t>
+          <t>957</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
+          <t>블록체인 관련 서울경제 보도에 대한 설명자료</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2606&amp;page=1</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>34467</t>
+          <t>55329</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -4755,22 +4755,22 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>955</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
+          <t>한국인터넷진흥원, 필리핀 사이버 위기 대응 역량 강화 지원</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2603&amp;page=1</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -4780,39 +4780,35 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>2945</t>
+          <t>34467</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H81" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:40.625220+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4822,27 +4818,27 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
+          <t>「2026 블록체인 밋업데이(BCMD)」 14회차 교육생 모집(~7.17)</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3699&amp;page=1</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>5048</t>
+          <t>2945</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -4869,32 +4865,32 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>954</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원 인사</t>
+          <t>제15회 정보보호의 날 기념식 개최 안내(서울 신라호텔, 7.8)</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3697&amp;page=1</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>145255</t>
+          <t>5048</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -4902,52 +4898,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-02 13:15:40.625220+09:00</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>954</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
+          <t>한국인터넷진흥원 인사</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2602&amp;page=1</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>26576</t>
+          <t>145255</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -4975,32 +4975,32 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>952</t>
+          <t>953</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
+          <t>한국인터넷진흥원, 특허법인·도메인등록기관과 케이(K)-브랜드 보호 협력</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2601&amp;page=1</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>34290</t>
+          <t>26576</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -5028,32 +5028,32 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>951</t>
+          <t>952</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
+          <t>한국인터넷진흥원, 국가 망 보안체계(N2SF) 도입 지원 본격화</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2600&amp;page=1</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>184573</t>
+          <t>34290</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -5081,32 +5081,32 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>14403</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>공지</t>
+          <t>951</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
+          <t>아피가(APIGA) 10년 성과, 글로벌 협력 확대로 잇는다</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2599&amp;page=1</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>6587</t>
+          <t>184573</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -5114,46 +5114,42 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="H87" t="inlineStr"/>
       <c r="I87" t="inlineStr">
         <is>
-          <t>공지사항</t>
+          <t>보도자료</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>2026-07-20 09:31:42.552965+09:00</t>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>14403</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>공지</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
+          <t>2026년 정보보호제품 성능평가 지원 공모 사업(~8/14)</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
+          <t>https://www.kisa.or.kr/401/form?postSeq=3682&amp;page=1</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -5163,7 +5159,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>51749</t>
+          <t>6587</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -5171,52 +5167,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr"/>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>보도자료</t>
+          <t>공지사항</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>2026-07-02 13:15:50.203272+09:00</t>
+          <t>2026-07-20 09:31:42.552965+09:00</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>949</t>
+          <t>950</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+          <t>음성스팸, 유선·인터넷전화 사업자와 함께 줄인다</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2598&amp;page=1</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>78439</t>
+          <t>51749</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -5244,55 +5244,108 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>949</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>한국 정보보호 기술, 인니 통신·금융 보안 수요와 만났다</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>https://www.kisa.or.kr/402/form?postSeq=2597&amp;page=1</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>78439</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:15:50.203272+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
           <t>38805</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr">
+      <c r="B91" t="inlineStr">
         <is>
           <t>공지</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr">
+      <c r="C91" t="inlineStr">
         <is>
           <t>[공유] 지능형 CCTV 성능시험 재개 안내 공지</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr">
+      <c r="D91" t="inlineStr">
         <is>
           <t>https://www.kisa.or.kr/401/form?postSeq=3677&amp;page=1</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr">
+      <c r="E91" t="inlineStr">
         <is>
           <t>2026-06-02</t>
         </is>
       </c>
-      <c r="F90" t="inlineStr">
+      <c r="F91" t="inlineStr">
         <is>
           <t>6525</t>
         </is>
       </c>
-      <c r="G90" t="inlineStr">
+      <c r="G91" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr">
+      <c r="H91" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr">
-        <is>
-          <t>공지사항</t>
-        </is>
-      </c>
-      <c r="J90" t="inlineStr">
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>공지사항</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
         <is>
           <t>2026-08-18 17:16:37.364015+09:00</t>
         </is>
       </c>
-      <c r="K90" t="inlineStr">
+      <c r="K91" t="inlineStr">
         <is>
           <t>2026-08-18 17:16:37.364015+09:00</t>
         </is>

</xml_diff>